<commit_message>
data: 2026-06-25 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-06-25.xlsx
+++ b/data/daily/2026-06-25.xlsx
@@ -426,12 +426,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="57" customWidth="1" min="3" max="3"/>
+    <col width="59" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="43" customWidth="1" min="6" max="6"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -502,7 +502,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -532,7 +532,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -562,7 +562,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -592,7 +592,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -622,7 +622,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -652,7 +652,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -682,7 +682,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -712,7 +712,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -742,7 +742,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>건강식품·영양제</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -766,6 +766,306 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>https://gift.kakao.com/product/5551542</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>물에 타먹는 발포형 무설탕 이온음료 요헤미티 워터 네가지 맛 4통(40정)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>요헤미티</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>34,000원</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/13372860</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+파인키위효소 1개월+저당견과류바</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>그레인온</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>43,900원</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/13180343</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)+프리미엄90 5포 추가증정</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>그레인온</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>20,000원</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/13180362</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>45,900원</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/11566779</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>아일로</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>65,900원</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/4965835</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>한끼통살</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>34,900원</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/12860133</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>익스트림</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>41,900원</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/7417420</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>한끼통살</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>20,000원</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/10848340</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CJ웰케어</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>8,900원</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/11190137</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>다이어트·이너뷰티</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>[운동선물/헬스] 삼대오백 모노 크레아틴 100서빙 운동 필수템</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>삼대오백</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>17,900원</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/6352718</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: kakao em dash 인코딩 오류 수정 / data: 2026-06-25 3개 플랫폼 수집 완료
</commit_message>
<xml_diff>
--- a/data/daily/2026-06-25.xlsx
+++ b/data/daily/2026-06-25.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="올리브영" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,32 +427,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -900,22 +889,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
+          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>아일로</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>65,900원</t>
+          <t>34,900원</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/4965835</t>
+          <t>https://gift.kakao.com/product/12860133</t>
         </is>
       </c>
     </row>
@@ -930,22 +919,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>아일로</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>34,900원</t>
+          <t>65,900원</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/12860133</t>
+          <t>https://gift.kakao.com/product/4965835</t>
         </is>
       </c>
     </row>
@@ -1092,32 +1081,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1330,6 +1319,360 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>상품명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>고려은단 비타민C1000 600정 (20개월분)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>고려은단</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>42,900원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000225938</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>덴프스</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>37,050원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000202658</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[호빵맨콜라보] 이너플로라 질유산균 60캡슐+호빵맨 스티커 / 이노시톨콜린 30포</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>뉴오리진</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38,900원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247265</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[서현PICK] 콜레올로지 PRO 600mg*30/60정 단품</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>17,400원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000175634</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[포켓몬 에디션] 덴마크 유산균이야기 30캡슐 1+1 (+꼬부기 러기지택) (60일분)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>덴프스</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>30,400원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000206861</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[헬로키티콜라보] 콜레올로지 컷팅 젤리 레몬/키위/석류 10+2포 기획</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>18,400원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000183645</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>고려은단 메가도스C 비타민C 3000mg 100포 (100일분)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>고려은단</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>25,900원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000225906</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[6월 올영픽/골라담기] CJ웰케어 건강루틴 가격혁명 10종 택 1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>씨제이웰케어</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5,900원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247861</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>프로뉴트리션</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>35,800원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000205496</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>건강식품</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>탄탄 더블컷 다이어트 젤리 3종 택1 (믹스베리맛/자두맛/애플유자맛)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>탄탄</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>9,900원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000213057</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>